<commit_message>
Mise à jour NHClima pour Rouen
</commit_message>
<xml_diff>
--- a/Remote/ug16/Données/03/dist_coûts.xlsx
+++ b/Remote/ug16/Données/03/dist_coûts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Mickaël\Documents\GitHub\ductaironline\Remote\ug16\Données\04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEE8698-25F1-451E-9F8B-DBCD40ECB6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EC7F2D-C1BC-441D-B024-5644DBB6D61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="86">
   <si>
     <t>id</t>
   </si>
@@ -272,16 +272,28 @@
     <t>Spécifique</t>
   </si>
   <si>
-    <t>NHCLIMA</t>
-  </si>
-  <si>
-    <t>DEBEAULIEU</t>
-  </si>
-  <si>
-    <t>NON DEFINI</t>
-  </si>
-  <si>
     <t>Fab NH</t>
+  </si>
+  <si>
+    <t>NH Clima</t>
+  </si>
+  <si>
+    <t>Debeaulieu</t>
+  </si>
+  <si>
+    <t>Taxe</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Affretement</t>
+  </si>
+  <si>
+    <t>Messagerie</t>
+  </si>
+  <si>
+    <t>Fournisseur 3 (non défini)</t>
   </si>
 </sst>
 </file>
@@ -635,7 +647,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AC25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -661,7 +673,7 @@
     <col min="24" max="24" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -740,8 +752,14 @@
       <c r="AA1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -749,7 +767,7 @@
         <v>20</v>
       </c>
       <c r="C2">
-        <v>1.8</v>
+        <v>1.85</v>
       </c>
       <c r="D2" s="1">
         <v>45748</v>
@@ -812,16 +830,22 @@
         <v>45</v>
       </c>
       <c r="Y2">
-        <v>2.25</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z2">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AA2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB2" t="s">
+        <v>83</v>
+      </c>
+      <c r="AC2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -892,16 +916,22 @@
         <v>40</v>
       </c>
       <c r="Y3">
-        <v>2.25</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z3">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AA3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB3" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -972,16 +1002,16 @@
         <v>35</v>
       </c>
       <c r="Y4">
-        <v>2.25</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z4">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AA4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1052,16 +1082,16 @@
         <v>30</v>
       </c>
       <c r="Y5">
-        <v>2.25</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z5">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="AA5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1096,7 +1126,7 @@
         <v>45748</v>
       </c>
       <c r="L6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="M6">
         <v>18</v>
@@ -1132,7 +1162,7 @@
         <v>25</v>
       </c>
       <c r="Y6">
-        <v>2.25</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z6">
         <v>60</v>
@@ -1141,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1209,7 +1239,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1277,7 +1307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1339,7 +1369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1389,16 +1419,16 @@
         <v>75</v>
       </c>
       <c r="Y10">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="Z10">
-        <v>0</v>
+        <v>9999</v>
       </c>
       <c r="AA10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+        <v>9999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1457,7 +1487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1504,16 +1534,16 @@
         <v>45748</v>
       </c>
       <c r="Y12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AA12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1560,7 +1590,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1607,7 +1637,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1654,7 +1684,7 @@
         <v>45748</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>

</xml_diff>